<commit_message>
updating benchmarks related files
</commit_message>
<xml_diff>
--- a/benchmarks_tests/FINAL_Benchmarks_for_paper/PyFock_scaling_behavior_GPU_CAO_old.xlsx
+++ b/benchmarks_tests/FINAL_Benchmarks_for_paper/PyFock_scaling_behavior_GPU_CAO_old.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manas/Documents/PyFock/benchmarks_tests/FINAL_Benchmarks_for_paper/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manas/Documents/PyFock__Benchmarks_Paper_IJQC/FINAL_Benchmarks_for_paper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC957A0E-DA30-A844-8568-79120B984C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4106BF-5F9D-6347-9C97-6BE8EF5AD700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1360" yWindow="760" windowWidth="28040" windowHeight="16960" xr2:uid="{580CF0B2-FD39-1547-AD8E-82680C382266}"/>
+    <workbookView xWindow="1360" yWindow="760" windowWidth="28040" windowHeight="16860" xr2:uid="{580CF0B2-FD39-1547-AD8E-82680C382266}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="def2-SVP" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -81,6 +81,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -123,10 +126,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -229,7 +233,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$B$19</c:f>
+              <c:f>'def2-SVP'!$B$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -264,7 +268,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$20:$A$28</c:f>
+              <c:f>'def2-SVP'!$A$20:$A$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -300,33 +304,33 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$20:$B$28</c:f>
+              <c:f>'def2-SVP'!$B$20:$B$28</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="1">
-                  <c:v>0.295609834603965</c:v>
+                  <c:v>0.11599999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.18141685805928232</c:v>
+                  <c:v>0.20153846153846156</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.46233239576506996</c:v>
+                  <c:v>0.46076923076923076</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.92976454365997996</c:v>
+                  <c:v>0.81133333333333335</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.8157904637356599</c:v>
+                  <c:v>1.526</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.1100739716716532</c:v>
+                  <c:v>3.2852941176470587</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.6650552651534003</c:v>
+                  <c:v>5.8793333333333333</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>14.484211621631376</c:v>
+                  <c:v>10.65</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -343,7 +347,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$C$19</c:f>
+              <c:f>'def2-SVP'!$C$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -378,7 +382,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$20:$A$28</c:f>
+              <c:f>'def2-SVP'!$A$20:$A$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -414,33 +418,33 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$C$20:$C$28</c:f>
+              <c:f>'def2-SVP'!$C$20:$C$28</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="1">
-                  <c:v>4.2427957803010903E-2</c:v>
+                  <c:v>2.6000000000000002E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.5847378725615774E-2</c:v>
+                  <c:v>5.0769230769230775E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1890870271107323</c:v>
+                  <c:v>0.15769230769230769</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.404987864072124</c:v>
+                  <c:v>0.34199999999999997</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.89636903262386669</c:v>
+                  <c:v>0.77066666666666672</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.172111773973</c:v>
+                  <c:v>1.8570588235294119</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.5270769301181</c:v>
+                  <c:v>3.7719999999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8.5446034903870629</c:v>
+                  <c:v>7.1312499999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -457,7 +461,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$D$19</c:f>
+              <c:f>'def2-SVP'!$D$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -492,7 +496,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$20:$A$28</c:f>
+              <c:f>'def2-SVP'!$A$20:$A$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -528,33 +532,33 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$D$20:$D$28</c:f>
+              <c:f>'def2-SVP'!$D$20:$D$28</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="1">
-                  <c:v>8.6814015824347696E-2</c:v>
+                  <c:v>5.2000000000000005E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.0823529967321764E-2</c:v>
+                  <c:v>8.8461538461538453E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.13197470793070692</c:v>
+                  <c:v>0.16692307692307692</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.26862757336348264</c:v>
+                  <c:v>0.26266666666666666</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.48043670977155334</c:v>
+                  <c:v>0.41266666666666668</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.99171357689534712</c:v>
+                  <c:v>0.7770588235294118</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.39670983701944</c:v>
+                  <c:v>1.0753333333333333</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.2431735377758688</c:v>
+                  <c:v>1.639375</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -981,7 +985,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$H$19</c:f>
+              <c:f>'def2-SVP'!$H$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1016,7 +1020,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$G$20:$G$28</c:f>
+              <c:f>'def2-SVP'!$G$20:$G$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -1052,33 +1056,33 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$H$20:$H$28</c:f>
+              <c:f>'def2-SVP'!$H$20:$H$28</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="1">
-                  <c:v>0.295609834603965</c:v>
+                  <c:v>0.11599999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.18141685805928232</c:v>
+                  <c:v>0.20153846153846156</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.46233239576506996</c:v>
+                  <c:v>0.46076923076923076</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.92976454365997996</c:v>
+                  <c:v>0.81133333333333335</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.8157904637356599</c:v>
+                  <c:v>1.526</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.1100739716716532</c:v>
+                  <c:v>3.2852941176470587</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.6650552651534003</c:v>
+                  <c:v>5.8793333333333333</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>14.484211621631376</c:v>
+                  <c:v>10.65</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1095,7 +1099,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$I$19</c:f>
+              <c:f>'def2-SVP'!$I$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1130,7 +1134,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$G$20:$G$28</c:f>
+              <c:f>'def2-SVP'!$G$20:$G$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -1166,33 +1170,33 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$I$20:$I$28</c:f>
+              <c:f>'def2-SVP'!$I$20:$I$28</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="1">
-                  <c:v>4.2427957803010903E-2</c:v>
+                  <c:v>2.6000000000000002E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.5847378725615774E-2</c:v>
+                  <c:v>5.0769230769230775E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1890870271107323</c:v>
+                  <c:v>0.15769230769230769</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.404987864072124</c:v>
+                  <c:v>0.34199999999999997</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.89636903262386669</c:v>
+                  <c:v>0.77066666666666672</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2.172111773973</c:v>
+                  <c:v>1.8570588235294119</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.5270769301181</c:v>
+                  <c:v>3.7719999999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8.5446034903870629</c:v>
+                  <c:v>7.1312499999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1209,7 +1213,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$J$19</c:f>
+              <c:f>'def2-SVP'!$J$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1244,7 +1248,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$G$20:$G$28</c:f>
+              <c:f>'def2-SVP'!$G$20:$G$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
@@ -1280,33 +1284,33 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$J$20:$J$28</c:f>
+              <c:f>'def2-SVP'!$J$20:$J$28</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="1">
-                  <c:v>8.6814015824347696E-2</c:v>
+                  <c:v>5.2000000000000005E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.0823529967321764E-2</c:v>
+                  <c:v>8.8461538461538453E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.13197470793070692</c:v>
+                  <c:v>0.16692307692307692</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.26862757336348264</c:v>
+                  <c:v>0.26266666666666666</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.48043670977155334</c:v>
+                  <c:v>0.41266666666666668</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.99171357689534712</c:v>
+                  <c:v>0.7770588235294118</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.39670983701944</c:v>
+                  <c:v>1.0753333333333333</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.2431735377758688</c:v>
+                  <c:v>1.639375</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3167,7 +3171,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B781A2DA-171B-7249-99BA-E5D7419364B8}">
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3259,23 +3263,29 @@
       <c r="B8">
         <v>125</v>
       </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+      <c r="C8" s="1">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.26</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.52</v>
+      </c>
       <c r="F8" s="1">
         <v>10</v>
       </c>
       <c r="G8">
         <f t="shared" ref="G8:G15" si="0">C8/F8</f>
-        <v>0</v>
+        <v>0.11599999999999999</v>
       </c>
       <c r="H8">
         <f t="shared" ref="H8:H15" si="1">D8/F8</f>
-        <v>0</v>
+        <v>2.6000000000000002E-2</v>
       </c>
       <c r="I8">
         <f t="shared" ref="I8:I15" si="2">E8/F8</f>
-        <v>0</v>
+        <v>5.2000000000000005E-2</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -3286,28 +3296,28 @@
         <v>250</v>
       </c>
       <c r="C9" s="1">
-        <v>2.3584191547706701</v>
+        <v>2.62</v>
       </c>
       <c r="D9" s="1">
-        <v>0.85601592343300503</v>
+        <v>0.66</v>
       </c>
       <c r="E9" s="1">
-        <v>0.66070588957518295</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="F9" s="1">
         <v>13</v>
       </c>
       <c r="G9">
         <f t="shared" si="0"/>
-        <v>0.18141685805928232</v>
+        <v>0.20153846153846156</v>
       </c>
       <c r="H9">
         <f t="shared" si="1"/>
-        <v>6.5847378725615774E-2</v>
+        <v>5.0769230769230775E-2</v>
       </c>
       <c r="I9">
         <f t="shared" si="2"/>
-        <v>5.0823529967321764E-2</v>
+        <v>8.8461538461538453E-2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -3318,28 +3328,28 @@
         <v>500</v>
       </c>
       <c r="C10" s="1">
-        <v>5.7691683680750403</v>
+        <v>5.99</v>
       </c>
       <c r="D10" s="1">
-        <v>2.1158297739457299</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="E10" s="1">
-        <v>2.0066158876288598</v>
+        <v>2.17</v>
       </c>
       <c r="F10" s="1">
         <v>13</v>
       </c>
       <c r="G10">
         <f t="shared" si="0"/>
-        <v>0.44378218215961851</v>
+        <v>0.46076923076923076</v>
       </c>
       <c r="H10">
         <f t="shared" si="1"/>
-        <v>0.16275613645736384</v>
+        <v>0.15769230769230769</v>
       </c>
       <c r="I10">
         <f t="shared" si="2"/>
-        <v>0.15435506827914305</v>
+        <v>0.16692307692307692</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -3350,28 +3360,28 @@
         <v>800</v>
       </c>
       <c r="C11" s="1">
-        <v>12.2090913550928</v>
+        <v>12.17</v>
       </c>
       <c r="D11" s="1">
-        <v>5.2523773421998996</v>
+        <v>5.13</v>
       </c>
       <c r="E11" s="1">
-        <v>3.9277749070897698</v>
+        <v>3.94</v>
       </c>
       <c r="F11" s="1">
         <v>15</v>
       </c>
       <c r="G11">
         <f t="shared" si="0"/>
-        <v>0.81393942367285332</v>
+        <v>0.81133333333333335</v>
       </c>
       <c r="H11">
         <f t="shared" si="1"/>
-        <v>0.35015848947999328</v>
+        <v>0.34199999999999997</v>
       </c>
       <c r="I11">
         <f t="shared" si="2"/>
-        <v>0.26185166047265135</v>
+        <v>0.26266666666666666</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -3382,28 +3392,28 @@
         <v>1175</v>
       </c>
       <c r="C12" s="1">
-        <v>23.0492668540682</v>
+        <v>22.89</v>
       </c>
       <c r="D12" s="1">
-        <v>11.764931902987801</v>
+        <v>11.56</v>
       </c>
       <c r="E12" s="1">
-        <v>6.2060886947438103</v>
+        <v>6.19</v>
       </c>
       <c r="F12" s="1">
         <v>15</v>
       </c>
       <c r="G12">
         <f t="shared" si="0"/>
-        <v>1.5366177902712133</v>
+        <v>1.526</v>
       </c>
       <c r="H12">
         <f t="shared" si="1"/>
-        <v>0.78432879353252005</v>
+        <v>0.77066666666666672</v>
       </c>
       <c r="I12">
         <f t="shared" si="2"/>
-        <v>0.41373924631625403</v>
+        <v>0.41266666666666668</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -3414,28 +3424,28 @@
         <v>1900</v>
       </c>
       <c r="C13" s="1">
-        <v>55.972384363878497</v>
+        <v>55.85</v>
       </c>
       <c r="D13" s="1">
-        <v>31.8730793460272</v>
+        <v>31.57</v>
       </c>
       <c r="E13" s="1">
-        <v>13.263924242928599</v>
+        <v>13.21</v>
       </c>
       <c r="F13" s="1">
         <v>17</v>
       </c>
       <c r="G13">
         <f t="shared" si="0"/>
-        <v>3.2924931978752059</v>
+        <v>3.2852941176470587</v>
       </c>
       <c r="H13">
         <f t="shared" si="1"/>
-        <v>1.8748870203545411</v>
+        <v>1.8570588235294119</v>
       </c>
       <c r="I13">
         <f t="shared" si="2"/>
-        <v>0.78023083781932934</v>
+        <v>0.7770588235294118</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -3446,28 +3456,28 @@
         <v>2500</v>
       </c>
       <c r="C14" s="1">
-        <v>88.581307347165406</v>
+        <v>88.19</v>
       </c>
       <c r="D14" s="1">
-        <v>57.356785830110297</v>
+        <v>56.58</v>
       </c>
       <c r="E14" s="1">
-        <v>16.1813672701828</v>
+        <v>16.13</v>
       </c>
       <c r="F14" s="1">
         <v>15</v>
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>5.9054204898110267</v>
+        <v>5.8793333333333333</v>
       </c>
       <c r="H14">
         <f t="shared" si="1"/>
-        <v>3.823785722007353</v>
+        <v>3.7719999999999998</v>
       </c>
       <c r="I14">
         <f t="shared" si="2"/>
-        <v>1.0787578180121866</v>
+        <v>1.0753333333333333</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -3478,28 +3488,28 @@
         <v>3475</v>
       </c>
       <c r="C15" s="1">
-        <v>171.51697664405199</v>
+        <v>170.4</v>
       </c>
       <c r="D15" s="1">
-        <v>114.241373233031</v>
+        <v>114.1</v>
       </c>
       <c r="E15" s="1">
-        <v>26.2381101583596</v>
+        <v>26.23</v>
       </c>
       <c r="F15" s="1">
         <v>16</v>
       </c>
       <c r="G15">
         <f t="shared" si="0"/>
-        <v>10.71981104025325</v>
+        <v>10.65</v>
       </c>
       <c r="H15">
         <f t="shared" si="1"/>
-        <v>7.1400858270644374</v>
+        <v>7.1312499999999996</v>
       </c>
       <c r="I15">
         <f t="shared" si="2"/>
-        <v>1.639881884897475</v>
+        <v>1.639375</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
@@ -3540,209 +3550,214 @@
       <c r="A21">
         <v>5</v>
       </c>
-      <c r="B21">
-        <v>0.295609834603965</v>
-      </c>
-      <c r="C21">
-        <v>4.2427957803010903E-2</v>
-      </c>
-      <c r="D21">
-        <v>8.6814015824347696E-2</v>
+      <c r="B21" s="3">
+        <v>0.11599999999999999</v>
+      </c>
+      <c r="C21" s="3">
+        <v>2.6000000000000002E-2</v>
+      </c>
+      <c r="D21" s="3">
+        <v>5.2000000000000005E-2</v>
       </c>
       <c r="G21">
         <v>125</v>
       </c>
-      <c r="H21">
-        <v>0.295609834603965</v>
-      </c>
-      <c r="I21">
-        <v>4.2427957803010903E-2</v>
-      </c>
-      <c r="J21">
-        <v>8.6814015824347696E-2</v>
+      <c r="H21" s="3">
+        <v>0.11599999999999999</v>
+      </c>
+      <c r="I21" s="3">
+        <v>2.6000000000000002E-2</v>
+      </c>
+      <c r="J21" s="3">
+        <v>5.2000000000000005E-2</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>10</v>
       </c>
-      <c r="B22">
-        <v>0.18141685805928232</v>
-      </c>
-      <c r="C22">
-        <v>6.5847378725615774E-2</v>
-      </c>
-      <c r="D22">
-        <v>5.0823529967321764E-2</v>
+      <c r="B22" s="3">
+        <v>0.20153846153846156</v>
+      </c>
+      <c r="C22" s="3">
+        <v>5.0769230769230775E-2</v>
+      </c>
+      <c r="D22" s="3">
+        <v>8.8461538461538453E-2</v>
       </c>
       <c r="G22">
         <v>250</v>
       </c>
-      <c r="H22">
-        <v>0.18141685805928232</v>
-      </c>
-      <c r="I22">
-        <v>6.5847378725615774E-2</v>
-      </c>
-      <c r="J22">
-        <v>5.0823529967321764E-2</v>
+      <c r="H22" s="3">
+        <v>0.20153846153846156</v>
+      </c>
+      <c r="I22" s="3">
+        <v>5.0769230769230775E-2</v>
+      </c>
+      <c r="J22" s="3">
+        <v>8.8461538461538453E-2</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>20</v>
       </c>
-      <c r="B23">
-        <v>0.46233239576506996</v>
-      </c>
-      <c r="C23">
-        <v>0.1890870271107323</v>
-      </c>
-      <c r="D23">
-        <v>0.13197470793070692</v>
+      <c r="B23" s="3">
+        <v>0.46076923076923076</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0.15769230769230769</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0.16692307692307692</v>
       </c>
       <c r="G23">
         <v>500</v>
       </c>
-      <c r="H23">
-        <v>0.46233239576506996</v>
-      </c>
-      <c r="I23">
-        <v>0.1890870271107323</v>
-      </c>
-      <c r="J23">
-        <v>0.13197470793070692</v>
+      <c r="H23" s="3">
+        <v>0.46076923076923076</v>
+      </c>
+      <c r="I23" s="3">
+        <v>0.15769230769230769</v>
+      </c>
+      <c r="J23" s="3">
+        <v>0.16692307692307692</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>32</v>
       </c>
-      <c r="B24">
-        <v>0.92976454365997996</v>
-      </c>
-      <c r="C24">
-        <v>0.404987864072124</v>
-      </c>
-      <c r="D24">
-        <v>0.26862757336348264</v>
+      <c r="B24" s="3">
+        <v>0.81133333333333335</v>
+      </c>
+      <c r="C24" s="3">
+        <v>0.34199999999999997</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0.26266666666666666</v>
       </c>
       <c r="G24">
         <v>800</v>
       </c>
-      <c r="H24">
-        <v>0.92976454365997996</v>
-      </c>
-      <c r="I24">
-        <v>0.404987864072124</v>
-      </c>
-      <c r="J24">
-        <v>0.26862757336348264</v>
+      <c r="H24" s="3">
+        <v>0.81133333333333335</v>
+      </c>
+      <c r="I24" s="3">
+        <v>0.34199999999999997</v>
+      </c>
+      <c r="J24" s="3">
+        <v>0.26266666666666666</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>47</v>
       </c>
-      <c r="B25">
-        <v>1.8157904637356599</v>
-      </c>
-      <c r="C25">
-        <v>0.89636903262386669</v>
-      </c>
-      <c r="D25">
-        <v>0.48043670977155334</v>
+      <c r="B25" s="3">
+        <v>1.526</v>
+      </c>
+      <c r="C25" s="3">
+        <v>0.77066666666666672</v>
+      </c>
+      <c r="D25" s="3">
+        <v>0.41266666666666668</v>
       </c>
       <c r="G25">
         <v>1175</v>
       </c>
-      <c r="H25">
-        <v>1.8157904637356599</v>
-      </c>
-      <c r="I25">
-        <v>0.89636903262386669</v>
-      </c>
-      <c r="J25">
-        <v>0.48043670977155334</v>
+      <c r="H25" s="3">
+        <v>1.526</v>
+      </c>
+      <c r="I25" s="3">
+        <v>0.77066666666666672</v>
+      </c>
+      <c r="J25" s="3">
+        <v>0.41266666666666668</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>76</v>
       </c>
-      <c r="B26">
-        <v>4.1100739716716532</v>
-      </c>
-      <c r="C26">
-        <v>2.172111773973</v>
-      </c>
-      <c r="D26">
-        <v>0.99171357689534712</v>
+      <c r="B26" s="3">
+        <v>3.2852941176470587</v>
+      </c>
+      <c r="C26" s="3">
+        <v>1.8570588235294119</v>
+      </c>
+      <c r="D26" s="3">
+        <v>0.7770588235294118</v>
       </c>
       <c r="G26">
         <v>1900</v>
       </c>
-      <c r="H26">
-        <v>4.1100739716716532</v>
-      </c>
-      <c r="I26">
-        <v>2.172111773973</v>
-      </c>
-      <c r="J26">
-        <v>0.99171357689534712</v>
+      <c r="H26" s="3">
+        <v>3.2852941176470587</v>
+      </c>
+      <c r="I26" s="3">
+        <v>1.8570588235294119</v>
+      </c>
+      <c r="J26" s="3">
+        <v>0.7770588235294118</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>100</v>
       </c>
-      <c r="B27">
-        <v>7.6650552651534003</v>
-      </c>
-      <c r="C27">
-        <v>4.5270769301181</v>
-      </c>
-      <c r="D27">
-        <v>1.39670983701944</v>
+      <c r="B27" s="3">
+        <v>5.8793333333333333</v>
+      </c>
+      <c r="C27" s="3">
+        <v>3.7719999999999998</v>
+      </c>
+      <c r="D27" s="3">
+        <v>1.0753333333333333</v>
       </c>
       <c r="G27">
         <v>2500</v>
       </c>
-      <c r="H27">
-        <v>7.6650552651534003</v>
-      </c>
-      <c r="I27">
-        <v>4.5270769301181</v>
-      </c>
-      <c r="J27">
-        <v>1.39670983701944</v>
+      <c r="H27" s="3">
+        <v>5.8793333333333333</v>
+      </c>
+      <c r="I27" s="3">
+        <v>3.7719999999999998</v>
+      </c>
+      <c r="J27" s="3">
+        <v>1.0753333333333333</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>139</v>
       </c>
-      <c r="B28">
-        <v>14.484211621631376</v>
-      </c>
-      <c r="C28">
-        <v>8.5446034903870629</v>
-      </c>
-      <c r="D28">
-        <v>2.2431735377758688</v>
+      <c r="B28" s="3">
+        <v>10.65</v>
+      </c>
+      <c r="C28" s="3">
+        <v>7.1312499999999996</v>
+      </c>
+      <c r="D28" s="3">
+        <v>1.639375</v>
       </c>
       <c r="G28">
         <v>3475</v>
       </c>
-      <c r="H28">
-        <v>14.484211621631376</v>
-      </c>
-      <c r="I28">
-        <v>8.5446034903870629</v>
-      </c>
-      <c r="J28">
-        <v>2.2431735377758688</v>
-      </c>
+      <c r="H28" s="3">
+        <v>10.65</v>
+      </c>
+      <c r="I28" s="3">
+        <v>7.1312499999999996</v>
+      </c>
+      <c r="J28" s="3">
+        <v>1.639375</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>